<commit_message>
commit before changing "IIeEE" to "II x 10^EE"
</commit_message>
<xml_diff>
--- a/optimized_benchmark_results/shaker_benchmark.xlsx
+++ b/optimized_benchmark_results/shaker_benchmark.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\afons\OneDrive - Universidade de Lisboa\Controlo de Plataforma Sismica\minimesa_data\optimized_benchmark_results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B96E7C7-A2C2-4F24-B057-A270A76C9A3B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{138CA3BD-7B6B-454C-BFB7-1D02893D9E76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-60" yWindow="-60" windowWidth="28920" windowHeight="16320" activeTab="1" xr2:uid="{40A5E321-79F6-4163-A8DE-342D0D4D7873}"/>
   </bookViews>
@@ -2985,6 +2985,817 @@
 </c:chartSpace>
 </file>
 
+<file path=xl/charts/chart12.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="pt-PT"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:autoTitleDeleted val="1"/>
+    <c:plotArea>
+      <c:layout>
+        <c:manualLayout>
+          <c:layoutTarget val="inner"/>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="0.17734249432788887"/>
+          <c:y val="3.529788079476457E-2"/>
+          <c:w val="0.81091179267250157"/>
+          <c:h val="0.6457875809406699"/>
+        </c:manualLayout>
+      </c:layout>
+      <c:lineChart>
+        <c:grouping val="standard"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Folha1!$K$7</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>OLI 3rd</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:solidFill>
+                <a:srgbClr val="00B0F0"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="00B0F0"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:srgbClr val="00B0F0"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:cat>
+            <c:strRef>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                  <c15:fullRef>
+                    <c15:sqref>Folha1!$J$8:$J$37</c15:sqref>
+                  </c15:fullRef>
+                </c:ext>
+              </c:extLst>
+              <c:f>(Folha1!$J$8,Folha1!$J$10,Folha1!$J$12,Folha1!$J$14,Folha1!$J$16,Folha1!$J$18,Folha1!$J$20,Folha1!$J$22,Folha1!$J$24,Folha1!$J$26,Folha1!$J$28,Folha1!$J$30,Folha1!$J$32,Folha1!$J$34,Folha1!$J$36)</c:f>
+              <c:strCache>
+                <c:ptCount val="15"/>
+                <c:pt idx="0">
+                  <c:v>El Centro (FN)</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>El Centro (FP)</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Erzikan (NS)</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Erzikan (EW)</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Kobe (NS)</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Kobe (EW)</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>L'Aquila</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>Newhall (FN)</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>Newhall (FP)</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>Rinaldi (FN)</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>Rinaldi (FP)</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>Sylmar (FN)</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>Sylmar (FP)</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>Tolmezzo</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>Average</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                  <c15:fullRef>
+                    <c15:sqref>Folha1!$K$8:$K$37</c15:sqref>
+                  </c15:fullRef>
+                </c:ext>
+              </c:extLst>
+              <c:f>(Folha1!$K$8,Folha1!$K$10,Folha1!$K$12,Folha1!$K$14,Folha1!$K$16,Folha1!$K$18,Folha1!$K$20,Folha1!$K$22,Folha1!$K$24,Folha1!$K$26,Folha1!$K$28,Folha1!$K$30,Folha1!$K$32,Folha1!$K$34,Folha1!$K$36)</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="15"/>
+                <c:pt idx="0">
+                  <c:v>-4.3089185078770313</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>-5.017728766960432</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>-5.4248121550723392</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>-5.1487416512809245</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>-4.7212463990471711</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>-4.7670038896078459</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>-4.3957739469155301</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>-4.8416375079047507</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>-4.6003262785189616</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>-4.4089353929735005</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>-4.1870866433571443</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>-4.3001622741327541</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>-5.0083309926200519</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>-2.7772835288524167</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>-3.840933642603702</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-DC63-4EF5-9EFF-99F2CBA012A4}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Folha1!$L$7</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>PID-F</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:srgbClr val="FF0000"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:cat>
+            <c:strRef>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                  <c15:fullRef>
+                    <c15:sqref>Folha1!$J$8:$J$37</c15:sqref>
+                  </c15:fullRef>
+                </c:ext>
+              </c:extLst>
+              <c:f>(Folha1!$J$8,Folha1!$J$10,Folha1!$J$12,Folha1!$J$14,Folha1!$J$16,Folha1!$J$18,Folha1!$J$20,Folha1!$J$22,Folha1!$J$24,Folha1!$J$26,Folha1!$J$28,Folha1!$J$30,Folha1!$J$32,Folha1!$J$34,Folha1!$J$36)</c:f>
+              <c:strCache>
+                <c:ptCount val="15"/>
+                <c:pt idx="0">
+                  <c:v>El Centro (FN)</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>El Centro (FP)</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Erzikan (NS)</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Erzikan (EW)</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Kobe (NS)</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Kobe (EW)</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>L'Aquila</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>Newhall (FN)</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>Newhall (FP)</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>Rinaldi (FN)</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>Rinaldi (FP)</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>Sylmar (FN)</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>Sylmar (FP)</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>Tolmezzo</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>Average</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                  <c15:fullRef>
+                    <c15:sqref>Folha1!$L$8:$L$37</c15:sqref>
+                  </c15:fullRef>
+                </c:ext>
+              </c:extLst>
+              <c:f>(Folha1!$L$8,Folha1!$L$10,Folha1!$L$12,Folha1!$L$14,Folha1!$L$16,Folha1!$L$18,Folha1!$L$20,Folha1!$L$22,Folha1!$L$24,Folha1!$L$26,Folha1!$L$28,Folha1!$L$30,Folha1!$L$32,Folha1!$L$34,Folha1!$L$36)</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="15"/>
+                <c:pt idx="0">
+                  <c:v>-4.2502636844309389</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>-4.8794260687941504</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>-5.6989700043360187</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>-5.3861581781239307</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>-4.5086383061657269</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>-4.6798537138889458</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>-4.7033348097384691</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>-4.8728952016351927</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>-5.1706962271689747</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>-4.7447274948966935</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>-4.2298847052128981</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>-4.7304870557820839</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>-5.3027706572402824</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>-3.5171264163912461</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>-4.3888535048526878</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-DC63-4EF5-9EFF-99F2CBA012A4}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="2"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Folha1!$M$7</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>LQI</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:solidFill>
+                <a:srgbClr val="FFC000"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="FFC000"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:srgbClr val="FFC000"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:cat>
+            <c:strRef>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                  <c15:fullRef>
+                    <c15:sqref>Folha1!$J$8:$J$37</c15:sqref>
+                  </c15:fullRef>
+                </c:ext>
+              </c:extLst>
+              <c:f>(Folha1!$J$8,Folha1!$J$10,Folha1!$J$12,Folha1!$J$14,Folha1!$J$16,Folha1!$J$18,Folha1!$J$20,Folha1!$J$22,Folha1!$J$24,Folha1!$J$26,Folha1!$J$28,Folha1!$J$30,Folha1!$J$32,Folha1!$J$34,Folha1!$J$36)</c:f>
+              <c:strCache>
+                <c:ptCount val="15"/>
+                <c:pt idx="0">
+                  <c:v>El Centro (FN)</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>El Centro (FP)</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Erzikan (NS)</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Erzikan (EW)</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Kobe (NS)</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Kobe (EW)</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>L'Aquila</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>Newhall (FN)</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>Newhall (FP)</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>Rinaldi (FN)</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>Rinaldi (FP)</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>Sylmar (FN)</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>Sylmar (FP)</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>Tolmezzo</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>Average</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                  <c15:fullRef>
+                    <c15:sqref>Folha1!$M$8:$M$37</c15:sqref>
+                  </c15:fullRef>
+                </c:ext>
+              </c:extLst>
+              <c:f>(Folha1!$M$8,Folha1!$M$10,Folha1!$M$12,Folha1!$M$14,Folha1!$M$16,Folha1!$M$18,Folha1!$M$20,Folha1!$M$22,Folha1!$M$24,Folha1!$M$26,Folha1!$M$28,Folha1!$M$30,Folha1!$M$32,Folha1!$M$34,Folha1!$M$36)</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="15"/>
+                <c:pt idx="0">
+                  <c:v>-4.9546770212133424</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>-5.519993057042849</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>-6.4168012260313771</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>-7.1530446749801762</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>-6.5114492834995561</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>-5.924453038607469</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>-6.3851027839668655</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>-6.0515870342213987</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>-5.79317412396815</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>-5.5718652059712115</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>-4.3645162531850881</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>-5.5100415205751654</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>-6.3665315444204138</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>-4.0584885673655968</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>-4.9536127119580806</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000002-DC63-4EF5-9EFF-99F2CBA012A4}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:marker val="1"/>
+        <c:smooth val="0"/>
+        <c:axId val="1230024880"/>
+        <c:axId val="1230026800"/>
+      </c:lineChart>
+      <c:catAx>
+        <c:axId val="1230024880"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="high"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="800" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1"/>
+                </a:solidFill>
+                <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="pt-PT"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1230026800"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="1230026800"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+          <c:max val="-2.5"/>
+          <c:min val="-8"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="800" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1"/>
+                    </a:solidFill>
+                    <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="pt-PT"/>
+                  <a:t>Acceleration Response Spectrum MSE (m s</a:t>
+                </a:r>
+                <a:r>
+                  <a:rPr lang="pt-PT" baseline="30000"/>
+                  <a:t>-2</a:t>
+                </a:r>
+                <a:r>
+                  <a:rPr lang="pt-PT"/>
+                  <a:t>)</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:layout>
+            <c:manualLayout>
+              <c:xMode val="edge"/>
+              <c:yMode val="edge"/>
+              <c:x val="1.2355920968811033E-2"/>
+              <c:y val="0.18498971108067039"/>
+            </c:manualLayout>
+          </c:layout>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="800" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="pt-PT"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="[=-3]&quot;10⁻³&quot;;[=-8]&quot;10⁻⁸&quot;" sourceLinked="0"/>
+        <c:majorTickMark val="cross"/>
+        <c:minorTickMark val="out"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:solidFill>
+              <a:schemeClr val="tx1"/>
+            </a:solidFill>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="800" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1"/>
+                </a:solidFill>
+                <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="pt-PT"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1230024880"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+        <c:majorUnit val="5"/>
+        <c:minorUnit val="1"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:solidFill>
+            <a:sysClr val="windowText" lastClr="000000"/>
+          </a:solidFill>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:layout>
+        <c:manualLayout>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="0.50355182575512458"/>
+          <c:y val="0.92081590851569173"/>
+          <c:w val="0.49644831430277098"/>
+          <c:h val="7.4286458754076759E-2"/>
+        </c:manualLayout>
+      </c:layout>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="800" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="pt-PT"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr sz="800">
+          <a:solidFill>
+            <a:schemeClr val="tx1"/>
+          </a:solidFill>
+          <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+          <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+        </a:defRPr>
+      </a:pPr>
+      <a:endParaRPr lang="pt-PT"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
@@ -9076,6 +9887,46 @@
 </cs:colorStyle>
 </file>
 
+<file path=xl/charts/colors12.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
 <file path=xl/charts/colors2.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
@@ -10429,6 +11280,522 @@
 </file>
 
 <file path=xl/charts/style11.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="227">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style12.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="227">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
@@ -15491,6 +16858,44 @@
     </xdr:graphicFrame>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>39688</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>145521</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>26</xdr:col>
+      <xdr:colOff>69006</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>3813</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="8" name="Gráfico 7">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9F270BDE-1B55-432C-B279-3EC3FD5AC7B4}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks/>
+        </xdr:cNvGraphicFramePr>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId9"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -16508,6 +17913,20 @@
     </row>
   </sheetData>
   <mergeCells count="25">
+    <mergeCell ref="D8:D11"/>
+    <mergeCell ref="E8:E9"/>
+    <mergeCell ref="E10:E11"/>
+    <mergeCell ref="D12:D15"/>
+    <mergeCell ref="E12:E13"/>
+    <mergeCell ref="E14:E15"/>
+    <mergeCell ref="D38:D39"/>
+    <mergeCell ref="E38:E39"/>
+    <mergeCell ref="D30:D33"/>
+    <mergeCell ref="E30:E31"/>
+    <mergeCell ref="E32:E33"/>
+    <mergeCell ref="D34:D37"/>
+    <mergeCell ref="E34:E35"/>
+    <mergeCell ref="E36:E37"/>
     <mergeCell ref="E24:E25"/>
     <mergeCell ref="D26:D29"/>
     <mergeCell ref="E26:E27"/>
@@ -16519,20 +17938,6 @@
     <mergeCell ref="D20:D23"/>
     <mergeCell ref="E20:E21"/>
     <mergeCell ref="E22:E23"/>
-    <mergeCell ref="D38:D39"/>
-    <mergeCell ref="E38:E39"/>
-    <mergeCell ref="D30:D33"/>
-    <mergeCell ref="E30:E31"/>
-    <mergeCell ref="E32:E33"/>
-    <mergeCell ref="D34:D37"/>
-    <mergeCell ref="E34:E35"/>
-    <mergeCell ref="E36:E37"/>
-    <mergeCell ref="D8:D11"/>
-    <mergeCell ref="E8:E9"/>
-    <mergeCell ref="E10:E11"/>
-    <mergeCell ref="D12:D15"/>
-    <mergeCell ref="E12:E13"/>
-    <mergeCell ref="E14:E15"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -17835,15 +19240,13 @@
     </row>
   </sheetData>
   <mergeCells count="32">
-    <mergeCell ref="A26:A29"/>
-    <mergeCell ref="B26:B27"/>
-    <mergeCell ref="B28:B29"/>
-    <mergeCell ref="A36:A37"/>
-    <mergeCell ref="A30:A33"/>
-    <mergeCell ref="B30:B31"/>
-    <mergeCell ref="B32:B33"/>
-    <mergeCell ref="A34:A35"/>
-    <mergeCell ref="B34:B35"/>
+    <mergeCell ref="D8:D11"/>
+    <mergeCell ref="D12:D15"/>
+    <mergeCell ref="D34:D35"/>
+    <mergeCell ref="D26:D29"/>
+    <mergeCell ref="D30:D33"/>
+    <mergeCell ref="D20:D21"/>
+    <mergeCell ref="D22:D25"/>
     <mergeCell ref="D36:D37"/>
     <mergeCell ref="D16:D19"/>
     <mergeCell ref="A8:A11"/>
@@ -17860,13 +19263,15 @@
     <mergeCell ref="A22:A25"/>
     <mergeCell ref="B22:B23"/>
     <mergeCell ref="B24:B25"/>
-    <mergeCell ref="D8:D11"/>
-    <mergeCell ref="D12:D15"/>
-    <mergeCell ref="D34:D35"/>
-    <mergeCell ref="D26:D29"/>
-    <mergeCell ref="D30:D33"/>
-    <mergeCell ref="D20:D21"/>
-    <mergeCell ref="D22:D25"/>
+    <mergeCell ref="A26:A29"/>
+    <mergeCell ref="B26:B27"/>
+    <mergeCell ref="B28:B29"/>
+    <mergeCell ref="A36:A37"/>
+    <mergeCell ref="A30:A33"/>
+    <mergeCell ref="B30:B31"/>
+    <mergeCell ref="B32:B33"/>
+    <mergeCell ref="A34:A35"/>
+    <mergeCell ref="B34:B35"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>